<commit_message>
docs:parte dos de BD
</commit_message>
<xml_diff>
--- a/Empresa Adoptfest/Normalizacion BD/BD Adoptafest - 1.xlsx
+++ b/Empresa Adoptfest/Normalizacion BD/BD Adoptafest - 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\adoptfest\Empresa Adoptfest\Normalizacion BD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{26846CA4-B804-4855-B73E-1DA445BD2C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2C41CF7-E884-442E-A08D-8B4FA3FD0885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{C45981E8-43C8-47A0-9373-D73F6CC0F80D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="85">
   <si>
     <t>ID_Mascota</t>
   </si>
@@ -325,6 +325,18 @@
   </si>
   <si>
     <t>n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eventos </t>
+  </si>
+  <si>
+    <t>ID_Evento - ID_Mascota</t>
+  </si>
+  <si>
+    <t>ID_Evento - ID_Organi</t>
+  </si>
+  <si>
+    <t>Organización</t>
   </si>
 </sst>
 </file>
@@ -406,7 +418,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -458,6 +470,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -606,7 +630,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -635,61 +659,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -702,14 +672,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -729,13 +693,91 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -761,21 +803,21 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>1404116</xdr:colOff>
-      <xdr:row>64</xdr:row>
+      <xdr:row>65</xdr:row>
       <xdr:rowOff>136071</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>1286494</xdr:colOff>
-      <xdr:row>72</xdr:row>
+      <xdr:row>73</xdr:row>
       <xdr:rowOff>156012</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="3" name="Conector recto 2">
+        <xdr:cNvPr id="2" name="Conector recto 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90E460CB-D238-EEC2-F97D-C06D189788C1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FAED2BEE-CB28-4220-A827-66EA9F09F794}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -783,8 +825,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="11312590" y="13285519"/>
-          <a:ext cx="1317313" cy="1529097"/>
+          <a:off x="12319766" y="14233071"/>
+          <a:ext cx="1253978" cy="1582041"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -811,21 +853,21 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>1395905</xdr:colOff>
-      <xdr:row>74</xdr:row>
+      <xdr:row>75</xdr:row>
       <xdr:rowOff>180647</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>16422</xdr:colOff>
-      <xdr:row>80</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>90324</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="5" name="Conector recto 4">
+        <xdr:cNvPr id="4" name="Conector recto 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{659EA543-7A89-ED01-72F7-426DC8AB0EDB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F8CD553B-6735-44A6-B966-2EC824D1A01C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -833,8 +875,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11306832" y="15240000"/>
-          <a:ext cx="1371271" cy="1059246"/>
+          <a:off x="12311555" y="16239797"/>
+          <a:ext cx="1277992" cy="1081252"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -861,21 +903,21 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>106746</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>82</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>106746</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:row>86</xdr:row>
       <xdr:rowOff>164224</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="7" name="Conector recto 6">
+        <xdr:cNvPr id="6" name="Conector recto 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F991E468-846C-00C4-410E-106C477EB9A9}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B1DE730-6FD6-42F5-B815-5CCC530FA731}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -883,8 +925,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12768427" y="16397780"/>
-          <a:ext cx="0" cy="919655"/>
+          <a:off x="13679871" y="17421225"/>
+          <a:ext cx="0" cy="954799"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -911,21 +953,21 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>172139</xdr:colOff>
-      <xdr:row>75</xdr:row>
+      <xdr:row>76</xdr:row>
       <xdr:rowOff>37110</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>12371</xdr:colOff>
-      <xdr:row>78</xdr:row>
+      <xdr:row>79</xdr:row>
       <xdr:rowOff>68856</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="9" name="Conector recto 8">
+        <xdr:cNvPr id="8" name="Conector recto 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1EBD47BC-F291-8A96-886B-C30A3516C325}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A633A163-94D1-4524-8D62-BB9966A3A9ED}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -933,8 +975,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="3734736" y="15252370"/>
-          <a:ext cx="1275167" cy="600772"/>
+          <a:off x="5039414" y="16286760"/>
+          <a:ext cx="1307082" cy="612771"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -961,21 +1003,21 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>195090</xdr:colOff>
-      <xdr:row>78</xdr:row>
+      <xdr:row>79</xdr:row>
       <xdr:rowOff>172139</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>1319729</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>85</xdr:row>
       <xdr:rowOff>57380</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="11" name="Conector recto 10">
+        <xdr:cNvPr id="10" name="Conector recto 9">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9D298F32-FF44-EEBB-AEE3-034963B0C1DD}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{363917EA-BD7E-430C-968E-8E1A0502630B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -983,8 +1025,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1" flipV="1">
-          <a:off x="3752620" y="15974458"/>
-          <a:ext cx="1124639" cy="1055783"/>
+          <a:off x="5062365" y="17002814"/>
+          <a:ext cx="1124639" cy="1066341"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -1009,32 +1051,232 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>160812</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>123701</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>23813</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>71437</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>49480</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>86591</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>750094</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>178594</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="15" name="Conector recto 14">
+        <xdr:cNvPr id="12" name="Conector recto 11">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D108799-71A7-CE13-798E-147250775F35}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B7DEA77A-0497-4EDD-A18D-E52463786840}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="12827825" y="13087597"/>
-          <a:ext cx="3191493" cy="148442"/>
+        <a:xfrm flipH="1">
+          <a:off x="18140363" y="13968412"/>
+          <a:ext cx="726281" cy="507207"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1000125</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>154781</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>11906</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="13" name="Conector recto 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{023AA91E-EA8A-41DE-85DA-2C8C591FBC58}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="9239250" y="16249650"/>
+          <a:ext cx="164306" cy="1183481"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>59531</xdr:colOff>
+      <xdr:row>83</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1071562</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>23812</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="14" name="Conector recto 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{92016F69-DDB9-4663-A511-8000FCBA3EFB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="10156031" y="17764125"/>
+          <a:ext cx="1012031" cy="1271587"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>214313</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>119062</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1762125</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>59531</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="16" name="Conector recto 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8ECE126C-741D-4FA0-A383-8FE2450DEBA8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="5081588" y="15016162"/>
+          <a:ext cx="3014662" cy="702469"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>345281</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>178594</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1440656</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="17" name="Conector recto 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D23DEB8E-8215-4363-8848-7F6EBEC4EDD2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="3745706" y="14275594"/>
+          <a:ext cx="1095375" cy="469106"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -1377,7 +1619,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00635D30-B81F-47E5-BAA0-A1F7C9D364B5}">
-  <dimension ref="B2:S88"/>
+  <dimension ref="B2:S92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
@@ -1397,7 +1639,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="12" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1667,27 +1909,27 @@
       </c>
     </row>
     <row r="10" spans="3:16" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="C10" s="29" t="s">
+      <c r="C10" s="11" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="11" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="39" t="s">
         <v>65</v>
       </c>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="12"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="41"/>
     </row>
     <row r="12" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="25"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="24"/>
     </row>
     <row r="14" spans="3:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C14" s="6" t="s">
@@ -1722,7 +1964,7 @@
       <c r="G15" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H15" s="22" t="s">
+      <c r="H15" s="10" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1796,28 +2038,28 @@
     </row>
     <row r="20" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="15"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="44"/>
     </row>
     <row r="22" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="19" t="s">
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="H23" s="20"/>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="21"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="30"/>
     </row>
     <row r="24" spans="3:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C24" s="7" t="s">
@@ -1995,12 +2237,12 @@
     </row>
     <row r="32" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C33" s="26" t="s">
+      <c r="C33" s="36" t="s">
         <v>71</v>
       </c>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="28"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="38"/>
     </row>
     <row r="34" spans="3:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C34" s="6" t="s">
@@ -2087,24 +2329,24 @@
       </c>
     </row>
     <row r="41" spans="3:11" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="C41" s="31" t="s">
+      <c r="C41" s="13" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="42" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C42" s="33" t="s">
+      <c r="C42" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="D42" s="35"/>
-      <c r="F42" s="33" t="s">
+      <c r="D42" s="33"/>
+      <c r="F42" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="G42" s="34"/>
-      <c r="H42" s="35"/>
-      <c r="J42" s="33" t="s">
+      <c r="G42" s="32"/>
+      <c r="H42" s="33"/>
+      <c r="J42" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="K42" s="35"/>
+      <c r="K42" s="33"/>
     </row>
     <row r="43" spans="3:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C43" s="6" t="s">
@@ -2246,19 +2488,19 @@
     </row>
     <row r="50" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="51" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C51" s="33" t="s">
+      <c r="C51" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="D51" s="34"/>
-      <c r="E51" s="35"/>
-      <c r="G51" s="33" t="s">
+      <c r="D51" s="32"/>
+      <c r="E51" s="33"/>
+      <c r="G51" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="H51" s="35"/>
-      <c r="J51" s="33" t="s">
+      <c r="H51" s="33"/>
+      <c r="J51" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="K51" s="35"/>
+      <c r="K51" s="33"/>
     </row>
     <row r="52" spans="2:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C52" s="7" t="s">
@@ -2296,7 +2538,7 @@
       <c r="G53" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H53" s="32" t="s">
+      <c r="H53" s="14" t="s">
         <v>13</v>
       </c>
       <c r="J53" s="5" t="s">
@@ -2398,150 +2640,200 @@
         <v>47</v>
       </c>
     </row>
-    <row r="58" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B59" s="36" t="s">
+    <row r="59" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B60" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="C59" s="37"/>
-      <c r="D59" s="37"/>
-      <c r="E59" s="37"/>
-      <c r="F59" s="37"/>
-      <c r="G59" s="37"/>
-      <c r="H59" s="37"/>
-      <c r="I59" s="37"/>
-      <c r="J59" s="37"/>
-      <c r="K59" s="37"/>
-      <c r="L59" s="37"/>
-      <c r="M59" s="37"/>
-      <c r="N59" s="37"/>
-      <c r="O59" s="37"/>
-      <c r="P59" s="37"/>
-      <c r="Q59" s="38"/>
-    </row>
-    <row r="60" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="39"/>
-      <c r="C60" s="40"/>
-      <c r="D60" s="40"/>
-      <c r="E60" s="40"/>
-      <c r="F60" s="40"/>
-      <c r="G60" s="40"/>
-      <c r="H60" s="40"/>
-      <c r="I60" s="40"/>
-      <c r="J60" s="40"/>
-      <c r="K60" s="40"/>
-      <c r="L60" s="40"/>
-      <c r="M60" s="40"/>
-      <c r="N60" s="40"/>
-      <c r="O60" s="40"/>
-      <c r="P60" s="40"/>
-      <c r="Q60" s="41"/>
-    </row>
-    <row r="62" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="63" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="P63" s="16" t="s">
+      <c r="C60" s="17"/>
+      <c r="D60" s="17"/>
+      <c r="E60" s="17"/>
+      <c r="F60" s="17"/>
+      <c r="G60" s="17"/>
+      <c r="H60" s="17"/>
+      <c r="I60" s="17"/>
+      <c r="J60" s="17"/>
+      <c r="K60" s="17"/>
+      <c r="L60" s="17"/>
+      <c r="M60" s="17"/>
+      <c r="N60" s="17"/>
+      <c r="O60" s="17"/>
+      <c r="P60" s="17"/>
+      <c r="Q60" s="18"/>
+    </row>
+    <row r="61" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="19"/>
+      <c r="C61" s="20"/>
+      <c r="D61" s="20"/>
+      <c r="E61" s="20"/>
+      <c r="F61" s="20"/>
+      <c r="G61" s="20"/>
+      <c r="H61" s="20"/>
+      <c r="I61" s="20"/>
+      <c r="J61" s="20"/>
+      <c r="K61" s="20"/>
+      <c r="L61" s="20"/>
+      <c r="M61" s="20"/>
+      <c r="N61" s="20"/>
+      <c r="O61" s="20"/>
+      <c r="P61" s="20"/>
+      <c r="Q61" s="21"/>
+    </row>
+    <row r="63" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="64" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P64" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="Q63" s="17"/>
-      <c r="R63" s="17"/>
-      <c r="S63" s="18"/>
-    </row>
-    <row r="64" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P64" s="42">
+      <c r="Q64" s="26"/>
+      <c r="R64" s="26"/>
+      <c r="S64" s="27"/>
+    </row>
+    <row r="65" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C65" s="45" t="s">
+        <v>81</v>
+      </c>
+      <c r="D65" s="46"/>
+      <c r="L65" s="15"/>
+      <c r="P65" s="15">
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="3:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="L65" t="s">
+    <row r="66" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D66" s="15">
+        <v>1</v>
+      </c>
+      <c r="L66" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="66" spans="3:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="L66" s="33" t="s">
+    <row r="67" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L67" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="M66" s="34"/>
-      <c r="N66" s="35"/>
-    </row>
-    <row r="73" spans="3:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="J73">
+      <c r="M67" s="32"/>
+      <c r="N67" s="33"/>
+    </row>
+    <row r="68" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="69" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E69" s="47" t="s">
+        <v>82</v>
+      </c>
+      <c r="F69" s="48"/>
+    </row>
+    <row r="70" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="E70" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="74" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F74">
         <v>1</v>
       </c>
-    </row>
-    <row r="74" spans="3:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F74" s="23" t="s">
+      <c r="J74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F75" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="G74" s="24"/>
-      <c r="H74" s="24"/>
-      <c r="I74" s="24"/>
-      <c r="J74" s="25"/>
-    </row>
-    <row r="75" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="F75" s="42">
+      <c r="G75" s="23"/>
+      <c r="H75" s="23"/>
+      <c r="I75" s="23"/>
+      <c r="J75" s="24"/>
+    </row>
+    <row r="76" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="F76" s="15">
         <v>1</v>
       </c>
-      <c r="J75">
+      <c r="G76">
         <v>1</v>
       </c>
-    </row>
-    <row r="78" spans="3:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="79" spans="3:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C79" s="33" t="s">
+      <c r="J76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="80" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C80" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="D79" s="35"/>
-      <c r="E79" s="42" t="s">
+      <c r="D80" s="33"/>
+      <c r="E80" s="15" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="80" spans="3:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="L80" s="33" t="s">
+    <row r="81" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L81" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="M80" s="34"/>
-      <c r="N80" s="35"/>
-    </row>
-    <row r="81" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="L81" t="s">
+      <c r="M81" s="32"/>
+      <c r="N81" s="33"/>
+    </row>
+    <row r="82" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="L82" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="85" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E85">
+    <row r="83" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H83" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="84" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G84" s="47" t="s">
+        <v>83</v>
+      </c>
+      <c r="H84" s="48"/>
+    </row>
+    <row r="86" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E86">
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="4:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D86" s="43" t="s">
+    <row r="87" spans="4:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D87" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="E86" s="44"/>
-    </row>
-    <row r="87" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="L87" s="42">
+      <c r="E87" s="35"/>
+    </row>
+    <row r="88" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L88" s="15">
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="L88" s="19" t="s">
+    <row r="89" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L89" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="M88" s="20"/>
-      <c r="N88" s="20"/>
-      <c r="O88" s="20"/>
-      <c r="P88" s="21"/>
+      <c r="M89" s="29"/>
+      <c r="N89" s="29"/>
+      <c r="O89" s="29"/>
+      <c r="P89" s="30"/>
+    </row>
+    <row r="91" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H92" s="49" t="s">
+        <v>84</v>
+      </c>
+      <c r="I92" s="50"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="B59:Q60"/>
-    <mergeCell ref="F74:J74"/>
-    <mergeCell ref="P63:S63"/>
-    <mergeCell ref="L88:P88"/>
-    <mergeCell ref="L80:N80"/>
-    <mergeCell ref="D86:E86"/>
-    <mergeCell ref="C79:D79"/>
-    <mergeCell ref="L66:N66"/>
+  <mergeCells count="24">
+    <mergeCell ref="L81:N81"/>
+    <mergeCell ref="G84:H84"/>
+    <mergeCell ref="D87:E87"/>
+    <mergeCell ref="L89:P89"/>
+    <mergeCell ref="H92:I92"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="G23:K23"/>
     <mergeCell ref="C33:F33"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="F42:H42"/>
@@ -2549,11 +2841,13 @@
     <mergeCell ref="C51:E51"/>
     <mergeCell ref="G51:H51"/>
     <mergeCell ref="J51:K51"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="B60:Q61"/>
+    <mergeCell ref="P64:S64"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="L67:N67"/>
+    <mergeCell ref="E69:F69"/>
+    <mergeCell ref="F75:J75"/>
+    <mergeCell ref="C80:D80"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>